<commit_message>
chore(data-release): publish site data 2026-08-16 02:00:19 UTC
</commit_message>
<xml_diff>
--- a/countries/tw/2026-2029.xlsx
+++ b/countries/tw/2026-2029.xlsx
@@ -42264,13 +42264,13 @@
         </is>
       </c>
       <c r="N252" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O252" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R252" t="n">
-        <v>0.12602508094667</v>
+        <v>0.1303707733931069</v>
       </c>
       <c r="S252" t="inlineStr">
         <is>
@@ -42423,10 +42423,10 @@
         </is>
       </c>
       <c r="N253" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O253" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U253" t="inlineStr">
         <is>
@@ -42657,13 +42657,13 @@
         </is>
       </c>
       <c r="N254" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O254" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R254" t="n">
-        <v>0.03476553957149517</v>
+        <v>0.03911123201793206</v>
       </c>
       <c r="S254" t="inlineStr">
         <is>
@@ -42816,10 +42816,10 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O255" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U255" t="inlineStr">
         <is>
@@ -43195,13 +43195,13 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="O257" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="R257" t="n">
-        <v>0.8865212590731267</v>
+        <v>0.8908669515195637</v>
       </c>
       <c r="S257" t="inlineStr">
         <is>
@@ -43340,13 +43340,13 @@
         </is>
       </c>
       <c r="N258" t="n">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="O258" t="n">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="R258" t="n">
-        <v>1.642671744753147</v>
+        <v>1.660054514538895</v>
       </c>
       <c r="S258" t="inlineStr">
         <is>
@@ -44996,13 +44996,13 @@
         </is>
       </c>
       <c r="N268" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O268" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R268" t="n">
-        <v>0.1347164658395438</v>
+        <v>0.1390621582859807</v>
       </c>
       <c r="S268" t="inlineStr">
         <is>
@@ -45155,10 +45155,10 @@
         </is>
       </c>
       <c r="N269" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O269" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="U269" t="inlineStr">
         <is>
@@ -45679,13 +45679,13 @@
         </is>
       </c>
       <c r="N272" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="O272" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="R272" t="n">
-        <v>0.460643399322311</v>
+        <v>0.4693347842151848</v>
       </c>
       <c r="S272" t="inlineStr">
         <is>
@@ -45824,13 +45824,13 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="O273" t="n">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="R273" t="n">
-        <v>0.5910141727154179</v>
+        <v>0.6214340198404762</v>
       </c>
       <c r="S273" t="inlineStr">
         <is>
@@ -45983,10 +45983,10 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="O274" t="n">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="U274" t="inlineStr">
         <is>
@@ -46721,7 +46721,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8343</v>
+        <v>8360</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-18 00:49:48 UTC
</commit_message>
<xml_diff>
--- a/countries/tw/2026-2029.xlsx
+++ b/countries/tw/2026-2029.xlsx
@@ -43195,13 +43195,13 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O257" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="R257" t="n">
-        <v>0.8908669515195637</v>
+        <v>0.8952126439660006</v>
       </c>
       <c r="S257" t="inlineStr">
         <is>
@@ -45795,22 +45795,22 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>D181</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Severe complicated COVID-19</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>新冠并发重症</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
@@ -45824,55 +45824,41 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="O273" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="R273" t="n">
-        <v>0.6214340198404762</v>
+        <v>0.004345692446436896</v>
       </c>
       <c r="S273" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
-      <c r="AA273" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO273" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP273" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ273" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS273" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR273" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS273" t="inlineStr"/>
       <c r="AT273" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU273" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV273" t="inlineStr">
@@ -45939,7 +45925,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -45988,98 +45974,23 @@
       <c r="O274" t="n">
         <v>143</v>
       </c>
+      <c r="R274" t="n">
+        <v>0.6214340198404762</v>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U274" t="inlineStr">
         <is>
           <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
         </is>
       </c>
-      <c r="V274" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
-      <c r="W274" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X274" t="inlineStr">
-        <is>
-          <t>新冠併發重症</t>
-        </is>
-      </c>
-      <c r="Y274" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z274" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA274" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB274" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC274" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD274" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE274" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF274" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG274" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH274" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI274" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ274" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK274" t="inlineStr">
-        <is>
-          <t>Taiwan NIDSS severe complicated COVID-19 series; a severe outcome category distinct from general COVID-19 notifications.</t>
-        </is>
-      </c>
-      <c r="AM274" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN274" t="b">
-        <v>1</v>
       </c>
       <c r="AO274" t="inlineStr">
         <is>
@@ -46173,7 +46084,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -46188,17 +46099,17 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>D210</t>
+          <t>D181</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Acute hepatitis C</t>
+          <t>Severe complicated COVID-19</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>急性丙型肝炎</t>
+          <t>新冠并发重症</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -46217,22 +46128,39 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="O275" t="n">
-        <v>16</v>
-      </c>
-      <c r="R275" t="n">
-        <v>0.06953107914299034</v>
-      </c>
-      <c r="S275" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>143</v>
       </c>
       <c r="U275" t="inlineStr">
         <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
+        </is>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
+        </is>
+      </c>
+      <c r="W275" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>新冠併發重症</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>notification</t>
         </is>
       </c>
       <c r="AA275" t="inlineStr">
@@ -46240,6 +46168,64 @@
           <t>monthly</t>
         </is>
       </c>
+      <c r="AB275" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC275" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD275" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE275" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF275" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG275" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH275" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI275" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ275" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK275" t="inlineStr">
+        <is>
+          <t>Taiwan NIDSS severe complicated COVID-19 series; a severe outcome category distinct from general COVID-19 notifications.</t>
+        </is>
+      </c>
+      <c r="AM275" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN275" t="b">
+        <v>1</v>
+      </c>
       <c r="AO275" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -46257,7 +46243,7 @@
       </c>
       <c r="AS275" t="inlineStr">
         <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
         </is>
       </c>
       <c r="AT275" t="n">
@@ -46332,7 +46318,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -46381,98 +46367,23 @@
       <c r="O276" t="n">
         <v>16</v>
       </c>
+      <c r="R276" t="n">
+        <v>0.06953107914299034</v>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U276" t="inlineStr">
         <is>
           <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
         </is>
       </c>
-      <c r="V276" t="inlineStr">
-        <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
-        </is>
-      </c>
-      <c r="W276" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X276" t="inlineStr">
-        <is>
-          <t>急性病毒性Ｃ型肝炎</t>
-        </is>
-      </c>
-      <c r="Y276" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z276" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA276" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB276" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC276" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD276" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE276" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF276" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG276" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH276" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI276" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ276" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK276" t="inlineStr">
-        <is>
-          <t>Acute hepatitis C, code 0705.</t>
-        </is>
-      </c>
-      <c r="AM276" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN276" t="b">
-        <v>1</v>
       </c>
       <c r="AO276" t="inlineStr">
         <is>
@@ -46538,6 +46449,240 @@
         </is>
       </c>
       <c r="BC276" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>tw</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>tw</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Taiwan, China</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Taiwan, China</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>D210</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Acute hepatitis C</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>急性丙型肝炎</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N277" t="n">
+        <v>16</v>
+      </c>
+      <c r="O277" t="n">
+        <v>16</v>
+      </c>
+      <c r="U277" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="W277" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>急性病毒性Ｃ型肝炎</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB277" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC277" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD277" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE277" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF277" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG277" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH277" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI277" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ277" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK277" t="inlineStr">
+        <is>
+          <t>Acute hepatitis C, code 0705.</t>
+        </is>
+      </c>
+      <c r="AM277" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN277" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO277" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP277" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ277" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS277" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="AT277" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU277" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV277" t="inlineStr">
+        <is>
+          <t>nidss_open_data</t>
+        </is>
+      </c>
+      <c r="AW277" t="inlineStr">
+        <is>
+          <t>Taiwan, China CDC NIDSS</t>
+        </is>
+      </c>
+      <c r="AX277" t="inlineStr">
+        <is>
+          <t>https://nidss.cdc.gov.tw/Home/Index</t>
+        </is>
+      </c>
+      <c r="AY277" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ277" t="inlineStr">
+        <is>
+          <t>nidss_open_data</t>
+        </is>
+      </c>
+      <c r="BA277" t="inlineStr">
+        <is>
+          <t>Taiwan, China CDC NIDSS</t>
+        </is>
+      </c>
+      <c r="BB277" t="inlineStr">
+        <is>
+          <t>https://nidss.cdc.gov.tw/Home/Index</t>
+        </is>
+      </c>
+      <c r="BC277" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -46659,7 +46804,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
@@ -46669,7 +46814,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11">
@@ -46721,7 +46866,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8360</v>
+        <v>8362</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-18 02:00:26 UTC
</commit_message>
<xml_diff>
--- a/countries/tw/2026-2029.xlsx
+++ b/countries/tw/2026-2029.xlsx
@@ -37834,13 +37834,13 @@
         </is>
       </c>
       <c r="N225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R225" t="n">
-        <v>0.008691384892873792</v>
+        <v>0.01303707733931069</v>
       </c>
       <c r="S225" t="inlineStr">
         <is>
@@ -39635,13 +39635,13 @@
         </is>
       </c>
       <c r="N236" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O236" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R236" t="n">
-        <v>0.08256815648230102</v>
+        <v>0.08691384892873792</v>
       </c>
       <c r="S236" t="inlineStr">
         <is>
@@ -39780,13 +39780,13 @@
         </is>
       </c>
       <c r="N237" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="O237" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R237" t="n">
-        <v>0.25205016189334</v>
+        <v>0.2563958543397769</v>
       </c>
       <c r="S237" t="inlineStr">
         <is>
@@ -40753,13 +40753,13 @@
         </is>
       </c>
       <c r="N243" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O243" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="R243" t="n">
-        <v>0.1347164658395438</v>
+        <v>0.1434078507324176</v>
       </c>
       <c r="S243" t="inlineStr">
         <is>
@@ -40898,13 +40898,13 @@
         </is>
       </c>
       <c r="N244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R244" t="n">
-        <v>0.004345692446436896</v>
+        <v>0.008691384892873792</v>
       </c>
       <c r="S244" t="inlineStr">
         <is>
@@ -42657,13 +42657,13 @@
         </is>
       </c>
       <c r="N254" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O254" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="R254" t="n">
-        <v>0.03911123201793206</v>
+        <v>0.05649400180367965</v>
       </c>
       <c r="S254" t="inlineStr">
         <is>
@@ -42816,10 +42816,10 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O255" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="U255" t="inlineStr">
         <is>
@@ -43050,13 +43050,13 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O256" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R256" t="n">
-        <v>0.04780261691080586</v>
+        <v>0.05214830935724275</v>
       </c>
       <c r="S256" t="inlineStr">
         <is>
@@ -43195,13 +43195,13 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>206</v>
+        <v>257</v>
       </c>
       <c r="O257" t="n">
-        <v>206</v>
+        <v>257</v>
       </c>
       <c r="R257" t="n">
-        <v>0.8952126439660006</v>
+        <v>1.116842958734282</v>
       </c>
       <c r="S257" t="inlineStr">
         <is>
@@ -43340,13 +43340,13 @@
         </is>
       </c>
       <c r="N258" t="n">
-        <v>382</v>
+        <v>423</v>
       </c>
       <c r="O258" t="n">
-        <v>382</v>
+        <v>423</v>
       </c>
       <c r="R258" t="n">
-        <v>1.660054514538895</v>
+        <v>1.838227904842807</v>
       </c>
       <c r="S258" t="inlineStr">
         <is>
@@ -43601,22 +43601,22 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>D058</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Scrub Typhus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>恙虫病</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L260" t="inlineStr">
@@ -43630,13 +43630,13 @@
         </is>
       </c>
       <c r="N260" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O260" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R260" t="n">
-        <v>0.01738276978574758</v>
+        <v>0.004345692446436896</v>
       </c>
       <c r="S260" t="inlineStr">
         <is>
@@ -43746,22 +43746,22 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>D068</t>
+          <t>D058</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Acute hepatitis B</t>
+          <t>Scrub Typhus</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>急性乙型肝炎</t>
+          <t>恙虫病</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
@@ -43775,55 +43775,41 @@
         </is>
       </c>
       <c r="N261" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O261" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R261" t="n">
-        <v>0.01738276978574758</v>
+        <v>0.02172846223218448</v>
       </c>
       <c r="S261" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
-        <is>
-          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
-        </is>
-      </c>
-      <c r="AA261" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO261" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP261" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ261" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS261" t="inlineStr">
-        <is>
-          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR261" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS261" t="inlineStr"/>
       <c r="AT261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU261" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV261" t="inlineStr">
@@ -43890,7 +43876,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -43939,98 +43925,23 @@
       <c r="O262" t="n">
         <v>4</v>
       </c>
+      <c r="R262" t="n">
+        <v>0.01738276978574758</v>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U262" t="inlineStr">
         <is>
           <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
         </is>
       </c>
-      <c r="V262" t="inlineStr">
-        <is>
-          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
-        </is>
-      </c>
-      <c r="W262" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X262" t="inlineStr">
-        <is>
-          <t>急性病毒性Ｂ型肝炎</t>
-        </is>
-      </c>
-      <c r="Y262" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z262" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA262" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB262" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC262" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD262" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE262" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF262" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG262" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH262" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI262" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ262" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK262" t="inlineStr">
-        <is>
-          <t>Acute hepatitis B, code 0703.</t>
-        </is>
-      </c>
-      <c r="AM262" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN262" t="b">
-        <v>1</v>
       </c>
       <c r="AO262" t="inlineStr">
         <is>
@@ -44124,7 +44035,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -44139,22 +44050,22 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>D105</t>
+          <t>D068</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Shigellosis</t>
+          <t>Acute hepatitis B</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>志贺菌病</t>
+          <t>急性乙型肝炎</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L263" t="inlineStr">
@@ -44173,17 +44084,34 @@
       <c r="O263" t="n">
         <v>4</v>
       </c>
-      <c r="R263" t="n">
-        <v>0.01738276978574758</v>
-      </c>
-      <c r="S263" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>SER_TW_SHIGELLOSIS_004</t>
+          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
+        </is>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>急性病毒性Ｂ型肝炎</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>notification</t>
         </is>
       </c>
       <c r="AA263" t="inlineStr">
@@ -44191,9 +44119,67 @@
           <t>monthly</t>
         </is>
       </c>
+      <c r="AB263" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC263" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD263" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE263" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF263" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG263" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH263" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI263" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ263" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK263" t="inlineStr">
+        <is>
+          <t>Acute hepatitis B, code 0703.</t>
+        </is>
+      </c>
+      <c r="AM263" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN263" t="b">
+        <v>1</v>
+      </c>
       <c r="AO263" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP263" t="inlineStr">
@@ -44203,12 +44189,12 @@
       </c>
       <c r="AQ263" t="inlineStr">
         <is>
-          <t>legacy_gap_fill</t>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS263" t="inlineStr">
         <is>
-          <t>SER_TW_SHIGELLOSIS_004</t>
+          <t>SER_TW_ACUTE_HEPATITIS_B_0703</t>
         </is>
       </c>
       <c r="AT263" t="n">
@@ -44216,7 +44202,7 @@
       </c>
       <c r="AU263" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV263" t="inlineStr">
@@ -44283,7 +44269,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -44332,98 +44318,23 @@
       <c r="O264" t="n">
         <v>4</v>
       </c>
+      <c r="R264" t="n">
+        <v>0.01738276978574758</v>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U264" t="inlineStr">
         <is>
           <t>SER_TW_SHIGELLOSIS_004</t>
         </is>
       </c>
-      <c r="V264" t="inlineStr">
-        <is>
-          <t>SER_TW_SHIGELLOSIS_004</t>
-        </is>
-      </c>
-      <c r="W264" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X264" t="inlineStr">
-        <is>
-          <t>桿菌性痢疾</t>
-        </is>
-      </c>
-      <c r="Y264" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z264" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA264" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB264" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC264" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD264" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE264" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF264" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG264" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH264" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI264" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ264" t="inlineStr">
-        <is>
-          <t>TW_NIDSS_004_current</t>
-        </is>
-      </c>
-      <c r="AK264" t="inlineStr">
-        <is>
-          <t>Taiwan NIDSS disease code 004, bacillary dysentery caused by Shigella; distinct from amoebiasis.</t>
-        </is>
-      </c>
-      <c r="AM264" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN264" t="b">
-        <v>1</v>
       </c>
       <c r="AO264" t="inlineStr">
         <is>
@@ -44517,7 +44428,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -44532,17 +44443,17 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>D106</t>
+          <t>D105</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Invasive pneumococcal disease</t>
+          <t>Shigellosis</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>侵袭性肺炎球菌病</t>
+          <t>志贺菌病</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -44561,41 +44472,130 @@
         </is>
       </c>
       <c r="N265" t="n">
+        <v>4</v>
+      </c>
+      <c r="O265" t="n">
+        <v>4</v>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>SER_TW_SHIGELLOSIS_004</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>SER_TW_SHIGELLOSIS_004</t>
+        </is>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>桿菌性痢疾</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB265" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC265" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD265" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE265" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF265" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG265" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH265" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI265" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ265" t="inlineStr">
+        <is>
+          <t>TW_NIDSS_004_current</t>
+        </is>
+      </c>
+      <c r="AK265" t="inlineStr">
+        <is>
+          <t>Taiwan NIDSS disease code 004, bacillary dysentery caused by Shigella; distinct from amoebiasis.</t>
+        </is>
+      </c>
+      <c r="AM265" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN265" t="b">
         <v>1</v>
       </c>
-      <c r="O265" t="n">
+      <c r="AO265" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP265" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ265" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS265" t="inlineStr">
+        <is>
+          <t>SER_TW_SHIGELLOSIS_004</t>
+        </is>
+      </c>
+      <c r="AT265" t="n">
         <v>1</v>
       </c>
-      <c r="R265" t="n">
-        <v>0.004345692446436896</v>
-      </c>
-      <c r="S265" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
-      <c r="AO265" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AP265" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR265" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS265" t="inlineStr"/>
-      <c r="AT265" t="n">
-        <v>0</v>
-      </c>
       <c r="AU265" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV265" t="inlineStr">
@@ -44677,17 +44677,17 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D106</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Invasive pneumococcal disease</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>侵袭性肺炎球菌病</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -44706,13 +44706,13 @@
         </is>
       </c>
       <c r="N266" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O266" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="R266" t="n">
-        <v>0.06518538669655344</v>
+        <v>0.008691384892873792</v>
       </c>
       <c r="S266" t="inlineStr">
         <is>
@@ -44822,17 +44822,17 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>D108</t>
+          <t>D107</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Listeriosis</t>
+          <t>Legionellosis</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>李斯特菌病</t>
+          <t>军团菌病</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -44851,13 +44851,13 @@
         </is>
       </c>
       <c r="N267" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="O267" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="R267" t="n">
-        <v>0.004345692446436896</v>
+        <v>0.07822246403586412</v>
       </c>
       <c r="S267" t="inlineStr">
         <is>
@@ -44967,22 +44967,22 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>D162</t>
+          <t>D108</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>HIV infection</t>
+          <t>Listeriosis</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>人类免疫缺乏病毒感染</t>
+          <t>李斯特菌病</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L268" t="inlineStr">
@@ -44996,55 +44996,41 @@
         </is>
       </c>
       <c r="N268" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="O268" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="R268" t="n">
-        <v>0.1390621582859807</v>
+        <v>0.008691384892873792</v>
       </c>
       <c r="S268" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
-        <is>
-          <t>SER_TW_HIV_044</t>
-        </is>
-      </c>
-      <c r="AA268" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO268" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP268" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ268" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS268" t="inlineStr">
-        <is>
-          <t>SER_TW_HIV_044</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR268" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS268" t="inlineStr"/>
       <c r="AT268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU268" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV268" t="inlineStr">
@@ -45111,7 +45097,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -45155,103 +45141,28 @@
         </is>
       </c>
       <c r="N269" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="O269" t="n">
-        <v>32</v>
+        <v>37</v>
+      </c>
+      <c r="R269" t="n">
+        <v>0.1607906205181651</v>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="U269" t="inlineStr">
         <is>
           <t>SER_TW_HIV_044</t>
         </is>
       </c>
-      <c r="V269" t="inlineStr">
-        <is>
-          <t>SER_TW_HIV_044</t>
-        </is>
-      </c>
-      <c r="W269" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X269" t="inlineStr">
-        <is>
-          <t>人類免疫缺乏病毒感染(含母子垂直感染及孕產婦疑似個案)</t>
-        </is>
-      </c>
-      <c r="Y269" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z269" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA269" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB269" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC269" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD269" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE269" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF269" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG269" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH269" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI269" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ269" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK269" t="inlineStr">
-        <is>
-          <t>NIDSS disease code 044, including source-specified vertical transmission and suspected maternal cases.</t>
-        </is>
-      </c>
-      <c r="AM269" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN269" t="b">
-        <v>1</v>
       </c>
       <c r="AO269" t="inlineStr">
         <is>
@@ -45345,7 +45256,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -45360,22 +45271,22 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>D165</t>
+          <t>D162</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Amebiasis</t>
+          <t>HIV infection</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>阿米巴病</t>
+          <t>人类免疫缺乏病毒感染</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
@@ -45389,41 +45300,130 @@
         </is>
       </c>
       <c r="N270" t="n">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="O270" t="n">
-        <v>9</v>
-      </c>
-      <c r="R270" t="n">
-        <v>0.03911123201793206</v>
-      </c>
-      <c r="S270" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>37</v>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>SER_TW_HIV_044</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>SER_TW_HIV_044</t>
+        </is>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>人類免疫缺乏病毒感染(含母子垂直感染及孕產婦疑似個案)</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB270" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC270" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD270" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE270" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF270" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG270" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH270" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI270" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ270" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK270" t="inlineStr">
+        <is>
+          <t>NIDSS disease code 044, including source-specified vertical transmission and suspected maternal cases.</t>
+        </is>
+      </c>
+      <c r="AM270" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN270" t="b">
+        <v>1</v>
       </c>
       <c r="AO270" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP270" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR270" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS270" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ270" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS270" t="inlineStr">
+        <is>
+          <t>SER_TW_HIV_044</t>
+        </is>
+      </c>
       <c r="AT270" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU270" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV270" t="inlineStr">
@@ -45505,22 +45505,22 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>D170</t>
+          <t>D165</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Complicated varicella</t>
+          <t>Amebiasis</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>水痘并发症</t>
+          <t>阿米巴病</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Parasitic</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -45534,13 +45534,13 @@
         </is>
       </c>
       <c r="N271" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="O271" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R271" t="n">
-        <v>0.004345692446436896</v>
+        <v>0.04345692446436896</v>
       </c>
       <c r="S271" t="inlineStr">
         <is>
@@ -45650,17 +45650,17 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>D172</t>
+          <t>D170</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Severe complicated influenza</t>
+          <t>Complicated varicella</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>流感并发重症</t>
+          <t>水痘并发症</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -45679,13 +45679,13 @@
         </is>
       </c>
       <c r="N272" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="O272" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="R272" t="n">
-        <v>0.4693347842151848</v>
+        <v>0.004345692446436896</v>
       </c>
       <c r="S272" t="inlineStr">
         <is>
@@ -45795,22 +45795,22 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D172</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Severe complicated influenza</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>流感并发重症</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
@@ -45824,13 +45824,13 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>1</v>
+        <v>137</v>
       </c>
       <c r="O273" t="n">
-        <v>1</v>
+        <v>137</v>
       </c>
       <c r="R273" t="n">
-        <v>0.004345692446436896</v>
+        <v>0.5953598651618548</v>
       </c>
       <c r="S273" t="inlineStr">
         <is>
@@ -45940,22 +45940,22 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>D181</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Severe complicated COVID-19</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>新冠并发重症</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -45969,55 +45969,41 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="O274" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="R274" t="n">
-        <v>0.6214340198404762</v>
+        <v>0.004345692446436896</v>
       </c>
       <c r="S274" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
-      <c r="AA274" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO274" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP274" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ274" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS274" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR274" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS274" t="inlineStr"/>
       <c r="AT274" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU274" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV274" t="inlineStr">
@@ -46084,7 +46070,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -46128,103 +46114,28 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>143</v>
+        <v>170</v>
       </c>
       <c r="O275" t="n">
-        <v>143</v>
+        <v>170</v>
+      </c>
+      <c r="R275" t="n">
+        <v>0.7387677158942723</v>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="U275" t="inlineStr">
         <is>
           <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
         </is>
       </c>
-      <c r="V275" t="inlineStr">
-        <is>
-          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
-        </is>
-      </c>
-      <c r="W275" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X275" t="inlineStr">
-        <is>
-          <t>新冠併發重症</t>
-        </is>
-      </c>
-      <c r="Y275" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z275" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA275" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB275" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC275" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD275" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE275" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF275" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG275" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH275" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI275" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ275" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK275" t="inlineStr">
-        <is>
-          <t>Taiwan NIDSS severe complicated COVID-19 series; a severe outcome category distinct from general COVID-19 notifications.</t>
-        </is>
-      </c>
-      <c r="AM275" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN275" t="b">
-        <v>1</v>
       </c>
       <c r="AO275" t="inlineStr">
         <is>
@@ -46318,7 +46229,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -46333,17 +46244,17 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>D210</t>
+          <t>D181</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Acute hepatitis C</t>
+          <t>Severe complicated COVID-19</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>急性丙型肝炎</t>
+          <t>新冠并发重症</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -46362,22 +46273,39 @@
         </is>
       </c>
       <c r="N276" t="n">
-        <v>16</v>
+        <v>170</v>
       </c>
       <c r="O276" t="n">
-        <v>16</v>
-      </c>
-      <c r="R276" t="n">
-        <v>0.06953107914299034</v>
-      </c>
-      <c r="S276" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>170</v>
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
+        </is>
+      </c>
+      <c r="W276" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>新冠併發重症</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>notification</t>
         </is>
       </c>
       <c r="AA276" t="inlineStr">
@@ -46385,6 +46313,64 @@
           <t>monthly</t>
         </is>
       </c>
+      <c r="AB276" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC276" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD276" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE276" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF276" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG276" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH276" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI276" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ276" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK276" t="inlineStr">
+        <is>
+          <t>Taiwan NIDSS severe complicated COVID-19 series; a severe outcome category distinct from general COVID-19 notifications.</t>
+        </is>
+      </c>
+      <c r="AM276" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN276" t="b">
+        <v>1</v>
+      </c>
       <c r="AO276" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -46402,7 +46388,7 @@
       </c>
       <c r="AS276" t="inlineStr">
         <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+          <t>SER_TW_SEVERE_COMPLICATED_COVID19_19SC</t>
         </is>
       </c>
       <c r="AT276" t="n">
@@ -46477,7 +46463,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -46526,98 +46512,23 @@
       <c r="O277" t="n">
         <v>16</v>
       </c>
+      <c r="R277" t="n">
+        <v>0.06953107914299034</v>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U277" t="inlineStr">
         <is>
           <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
         </is>
       </c>
-      <c r="V277" t="inlineStr">
-        <is>
-          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
-        </is>
-      </c>
-      <c r="W277" t="inlineStr">
-        <is>
-          <t>SRC_TW_NIDSS</t>
-        </is>
-      </c>
-      <c r="X277" t="inlineStr">
-        <is>
-          <t>急性病毒性Ｃ型肝炎</t>
-        </is>
-      </c>
-      <c r="Y277" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z277" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA277" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB277" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC277" t="inlineStr">
-        <is>
-          <t>country:TW:national</t>
-        </is>
-      </c>
-      <c r="AD277" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE277" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF277" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG277" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH277" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI277" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ277" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
-        </is>
-      </c>
-      <c r="AK277" t="inlineStr">
-        <is>
-          <t>Acute hepatitis C, code 0705.</t>
-        </is>
-      </c>
-      <c r="AM277" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN277" t="b">
-        <v>1</v>
       </c>
       <c r="AO277" t="inlineStr">
         <is>
@@ -46683,6 +46594,240 @@
         </is>
       </c>
       <c r="BC277" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>tw</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>tw</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Taiwan, China</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Taiwan, China</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>D210</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Acute hepatitis C</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>急性丙型肝炎</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N278" t="n">
+        <v>16</v>
+      </c>
+      <c r="O278" t="n">
+        <v>16</v>
+      </c>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t>SRC_TW_NIDSS</t>
+        </is>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>急性病毒性Ｃ型肝炎</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA278" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB278" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC278" t="inlineStr">
+        <is>
+          <t>country:TW:national</t>
+        </is>
+      </c>
+      <c r="AD278" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE278" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF278" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG278" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH278" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI278" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ278" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.10</t>
+        </is>
+      </c>
+      <c r="AK278" t="inlineStr">
+        <is>
+          <t>Acute hepatitis C, code 0705.</t>
+        </is>
+      </c>
+      <c r="AM278" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN278" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO278" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP278" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ278" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS278" t="inlineStr">
+        <is>
+          <t>SER_TW_ACUTE_HEPATITIS_C_0705</t>
+        </is>
+      </c>
+      <c r="AT278" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU278" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV278" t="inlineStr">
+        <is>
+          <t>nidss_open_data</t>
+        </is>
+      </c>
+      <c r="AW278" t="inlineStr">
+        <is>
+          <t>Taiwan, China CDC NIDSS</t>
+        </is>
+      </c>
+      <c r="AX278" t="inlineStr">
+        <is>
+          <t>https://nidss.cdc.gov.tw/Home/Index</t>
+        </is>
+      </c>
+      <c r="AY278" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ278" t="inlineStr">
+        <is>
+          <t>nidss_open_data</t>
+        </is>
+      </c>
+      <c r="BA278" t="inlineStr">
+        <is>
+          <t>Taiwan, China CDC NIDSS</t>
+        </is>
+      </c>
+      <c r="BB278" t="inlineStr">
+        <is>
+          <t>https://nidss.cdc.gov.tw/Home/Index</t>
+        </is>
+      </c>
+      <c r="BC278" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -46804,7 +46949,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
@@ -46814,7 +46959,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11">
@@ -46866,7 +47011,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8362</v>
+        <v>8534</v>
       </c>
     </row>
     <row r="16">

</xml_diff>